<commit_message>
updated open encounters exclusion criteria
</commit_message>
<xml_diff>
--- a/open_encounters_exclusion.xlsx
+++ b/open_encounters_exclusion.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kweons01\Desktop\Strategic Initiatives - So Youn\MSHS Ambulatory Reporting\server-files-upload\Mapping Files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kweons01\Desktop\Strategic Initiatives - So Youn\Github\server-upload\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19368" windowHeight="9192" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19368" windowHeight="9192"/>
   </bookViews>
   <sheets>
     <sheet name="Department" sheetId="2" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="115">
   <si>
     <t>DEPARTMENT</t>
   </si>
@@ -348,6 +348,24 @@
   </si>
   <si>
     <t>PRC_ID</t>
+  </si>
+  <si>
+    <t>2360 AMSTERDAM AVE CARDIOLOGY</t>
+  </si>
+  <si>
+    <t>440 W 114TH IAM DENTAL</t>
+  </si>
+  <si>
+    <t>2360 AMSTRDM SURG BARI</t>
+  </si>
+  <si>
+    <t>2360 AMSTRDAM SURG VAS</t>
+  </si>
+  <si>
+    <t>718 TEANECK ROAD SURG COLORECTAL</t>
+  </si>
+  <si>
+    <t>355 BARD AVE CARDIO SURG</t>
   </si>
 </sst>
 </file>
@@ -1173,7 +1191,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="31.6640625" bestFit="1" customWidth="1"/>
@@ -1214,8 +1232,75 @@
         <v>34</v>
       </c>
     </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B4">
+        <v>8109003</v>
+      </c>
+      <c r="C4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B5">
+        <v>8808068</v>
+      </c>
+      <c r="C5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B6">
+        <v>8109001</v>
+      </c>
+      <c r="C6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>112</v>
+      </c>
+      <c r="B7">
+        <v>8109002</v>
+      </c>
+      <c r="C7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B8">
+        <v>8303002</v>
+      </c>
+      <c r="C8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>114</v>
+      </c>
+      <c r="B9">
+        <v>8846001</v>
+      </c>
+      <c r="C9" t="s">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>